<commit_message>
chore: back up the Macro Tracker only before big system changes
Routine data runs (P0-P9) no longer take a workbook backup; the Update Log
already records every old -> new value. Backups are taken only before
structural, formula, threshold or source changes, and only the newest one
is kept. backups/ is now gitignored.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Macro_Tracker_v5.xlsx
+++ b/Macro_Tracker_v5.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/8d1bd21a83edf255/Desktop/Trading System/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="11_AC2D57271251B1C837B53BDED290A7124F3F60CB" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="11_07BBB4D6B1A3B2E06750235655848FBF97FA3FEE" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-38520" yWindow="-7095" windowWidth="38640" windowHeight="21120" tabRatio="500" activeTab="9" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -3557,7 +3557,7 @@
     <t>Work on the newest Macro_Tracker_v*.xlsx in OneDrive › Desktop › Trading System. If it is open/locked in Excel, do NOT overwrite it: stop and report the planned changes instead.</t>
   </si>
   <si>
-    <t>Back up first: copy it to backups/&lt;file&gt;_backup_&lt;YYYY-MM-DD_HHMM&gt;_&lt;prompt ID&gt;.xlsx.</t>
+    <t>Back up ONLY before a big change to the system — new or removed sheets/columns, layout, formulas, thresholds or data sources: copy the workbook to backups/&lt;file&gt;_backup_before-&lt;change&gt;_&lt;YYYY-MM-DD&gt;.xlsx and keep only the newest one (delete older backups). Routine data runs (P0–P9) take no backup — the Update Log already records every old → new value.</t>
   </si>
   <si>
     <t>Write ONLY cells whose Sources row says “Claude” (blue input cells). Never write cells marked “User”: Bias N/Q, User bias, User read, Compare, Journal, Guide thresholds, Events “User notes”, Calendar settings. “Claude drafts → User confirms” cells: put the draft in the note cell and leave the value unless it is empty.</t>
@@ -3611,7 +3611,7 @@
     <t>Everything below, in order. P5 only on Sundays, P6 only on the first run of the month.</t>
   </si>
   <si>
-    <t>Workbook: the newest Macro_Tracker_v*.xlsx in OneDrive › Desktop › Trading System (on the User’s computer; a copy may also live in the cloud later). Before starting, read the workbook’s Prompts sheet (UPDATE RULES) and Sources sheet (one fixed source per input + who fills each cell) and follow both exactly. Run the Macro Tracker FULL CYCLE for today. Do these prompts from the Prompts sheet in this order, as one run with one backup and one Update Log row: (1) P1 Events; (2) P2 Markets; (3) P3 Macro data — only for indicators with a new release since the last Update Log row; (4) P4 Country deep-dive for every currency that had a central-bank decision, central-bank speech, budget or tier-1 release since the last run, or whose Hub “Last checked” is older than 7 days; (5) if today is Sunday, P5 Key levels; (6) if this is the first run this month, P6 Who holds what; (7) P7 AI bias — always last. Finish with a 5-line summary: what changed, which Scorecard stances or FINAL BIAS values flipped, where the AI bias now disagrees with the model or the User bias, the next 3 high-impact events, and anything NOT UPDATED.</t>
+    <t>Workbook: the newest Macro_Tracker_v*.xlsx in OneDrive › Desktop › Trading System (on the User’s computer; a copy may also live in the cloud later). Before starting, read the workbook’s Prompts sheet (UPDATE RULES) and Sources sheet (one fixed source per input + who fills each cell) and follow both exactly. Run the Macro Tracker FULL CYCLE for today. Do these prompts from the Prompts sheet in this order, as one run with one Update Log row (no backup — routine run): (1) P1 Events; (2) P2 Markets; (3) P3 Macro data — only for indicators with a new release since the last Update Log row; (4) P4 Country deep-dive for every currency that had a central-bank decision, central-bank speech, budget or tier-1 release since the last run, or whose Hub “Last checked” is older than 7 days; (5) if today is Sunday, P5 Key levels; (6) if this is the first run this month, P6 Who holds what; (7) P7 AI bias — always last. Finish with a 5-line summary: what changed, which Scorecard stances or FINAL BIAS values flipped, where the AI bias now disagrees with the model or the User bias, the next 3 high-impact events, and anything NOT UPDATED.</t>
   </si>
   <si>
     <t>P1</t>
@@ -3779,18 +3779,18 @@
     <numFmt numFmtId="168" formatCode="0&quot; bp&quot;;\-0&quot; bp&quot;"/>
     <numFmt numFmtId="169" formatCode="0.0\%;\-0.0\%"/>
     <numFmt numFmtId="170" formatCode="\+0.00;\-0.00;0.00"/>
-    <numFmt numFmtId="172" formatCode="ddd\ d\-mmm\-yy"/>
-    <numFmt numFmtId="173" formatCode="d\-mmm\ hh:mm"/>
-    <numFmt numFmtId="174" formatCode="d"/>
-    <numFmt numFmtId="175" formatCode="\+0&quot; bp&quot;;\-0&quot; bp&quot;;0&quot; bp&quot;"/>
-    <numFmt numFmtId="176" formatCode="\+0.00&quot; pp&quot;;\-0.00&quot; pp&quot;;0.00&quot; pp&quot;"/>
-    <numFmt numFmtId="177" formatCode="0&quot; bp&quot;"/>
-    <numFmt numFmtId="178" formatCode="0.0&quot;%&quot;"/>
-    <numFmt numFmtId="179" formatCode="ddd\ d\-mmm\-yy\ hh:mm"/>
-    <numFmt numFmtId="180" formatCode="0.00;[Red]\-0.00"/>
-    <numFmt numFmtId="181" formatCode="dddd\ d\ mmm"/>
-    <numFmt numFmtId="182" formatCode="ddd\ d\ mmm\ yyyy"/>
-    <numFmt numFmtId="183" formatCode="dddd\ d\ mmmm\ yyyy"/>
+    <numFmt numFmtId="171" formatCode="ddd\ d\-mmm\-yy"/>
+    <numFmt numFmtId="172" formatCode="d\-mmm\ hh:mm"/>
+    <numFmt numFmtId="173" formatCode="d"/>
+    <numFmt numFmtId="174" formatCode="\+0&quot; bp&quot;;\-0&quot; bp&quot;;0&quot; bp&quot;"/>
+    <numFmt numFmtId="175" formatCode="\+0.00&quot; pp&quot;;\-0.00&quot; pp&quot;;0.00&quot; pp&quot;"/>
+    <numFmt numFmtId="176" formatCode="0&quot; bp&quot;"/>
+    <numFmt numFmtId="177" formatCode="0.0&quot;%&quot;"/>
+    <numFmt numFmtId="178" formatCode="ddd\ d\-mmm\-yy\ hh:mm"/>
+    <numFmt numFmtId="179" formatCode="0.00;[Red]\-0.00"/>
+    <numFmt numFmtId="180" formatCode="dddd\ d\ mmm"/>
+    <numFmt numFmtId="181" formatCode="ddd\ d\ mmm\ yyyy"/>
+    <numFmt numFmtId="182" formatCode="dddd\ d\ mmmm\ yyyy"/>
   </numFmts>
   <fonts count="116" x14ac:knownFonts="1">
     <font>
@@ -5530,7 +5530,7 @@
     <xf numFmtId="0" fontId="48" fillId="18" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="172" fontId="47" fillId="18" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="171" fontId="47" fillId="18" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="20" fontId="47" fillId="18" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -5539,7 +5539,7 @@
     <xf numFmtId="0" fontId="54" fillId="19" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="173" fontId="54" fillId="19" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="172" fontId="54" fillId="19" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="20" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -5576,7 +5576,7 @@
     <xf numFmtId="0" fontId="74" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="174" fontId="18" fillId="0" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="173" fontId="18" fillId="0" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="75" fillId="31" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -5720,10 +5720,10 @@
     <xf numFmtId="2" fontId="98" fillId="52" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="175" fontId="100" fillId="51" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="174" fontId="100" fillId="51" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="176" fontId="100" fillId="51" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="175" fontId="100" fillId="51" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="166" fontId="102" fillId="51" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -5760,11 +5760,11 @@
     <xf numFmtId="0" fontId="18" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
-    <xf numFmtId="177" fontId="102" fillId="51" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="176" fontId="102" fillId="51" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="18" xfId="0" applyBorder="1"/>
-    <xf numFmtId="178" fontId="102" fillId="51" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="177" fontId="102" fillId="51" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="49" fontId="102" fillId="51" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -5826,7 +5826,7 @@
     <xf numFmtId="0" fontId="110" fillId="58" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="179" fontId="114" fillId="61" borderId="29" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="178" fontId="114" fillId="61" borderId="29" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="114" fillId="61" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -5908,7 +5908,7 @@
     <xf numFmtId="40" fontId="98" fillId="61" borderId="32" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="180" fontId="100" fillId="51" borderId="32" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="179" fontId="100" fillId="51" borderId="32" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="1" fontId="100" fillId="51" borderId="32" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -5936,7 +5936,7 @@
     <xf numFmtId="0" fontId="64" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="181" fontId="71" fillId="28" borderId="31" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="180" fontId="71" fillId="28" borderId="31" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="20" fillId="29" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -5952,7 +5952,7 @@
     <xf numFmtId="0" fontId="70" fillId="30" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="182" fontId="18" fillId="29" borderId="29" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="181" fontId="18" fillId="29" borderId="29" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="22" xfId="0" applyBorder="1"/>
@@ -5970,7 +5970,7 @@
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
     <xf numFmtId="0" fontId="67" fillId="0" borderId="31" xfId="0" applyFont="1"/>
-    <xf numFmtId="183" fontId="18" fillId="29" borderId="29" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="182" fontId="18" fillId="29" borderId="29" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="88" fillId="0" borderId="31" xfId="0" applyFont="1" applyAlignment="1">
@@ -6002,12 +6002,12 @@
     <xf numFmtId="0" fontId="90" fillId="50" borderId="31" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="19" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="26" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="27" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="92" fillId="0" borderId="31" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="19" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="26" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="27" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="16" fillId="0" borderId="31" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
@@ -23026,7 +23026,7 @@
       </c>
       <c r="H6" s="239"/>
     </row>
-    <row r="7" spans="1:8" ht="36" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:8" ht="36" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="238">
         <v>46286.802083333343</v>
       </c>
@@ -27530,8 +27530,8 @@
   </sheetData>
   <mergeCells count="30">
     <mergeCell ref="A4:K4"/>
+    <mergeCell ref="D5:E5"/>
     <mergeCell ref="A6:C6"/>
-    <mergeCell ref="D5:E5"/>
     <mergeCell ref="M27:AA28"/>
     <mergeCell ref="H5:I5"/>
     <mergeCell ref="M9:AA9"/>
@@ -28493,7 +28493,7 @@
       </c>
     </row>
     <row r="2" spans="1:10" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="304" t="s">
+      <c r="A2" s="307" t="s">
         <v>354</v>
       </c>
       <c r="B2" s="273"/>
@@ -29999,7 +29999,7 @@
       </c>
       <c r="B75" s="188"/>
       <c r="C75" s="294"/>
-      <c r="D75" s="305"/>
+      <c r="D75" s="304"/>
       <c r="F75" s="213" t="s">
         <v>440</v>
       </c>
@@ -30017,8 +30017,8 @@
     <row r="76" spans="1:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A76" s="215"/>
       <c r="B76" s="215"/>
-      <c r="C76" s="306"/>
-      <c r="D76" s="307"/>
+      <c r="C76" s="305"/>
+      <c r="D76" s="306"/>
       <c r="F76" s="219" t="s">
         <v>441</v>
       </c>
@@ -30062,6 +30062,9 @@
   </sheetData>
   <mergeCells count="58">
     <mergeCell ref="C75:D76"/>
+    <mergeCell ref="A2:J2"/>
+    <mergeCell ref="C53:D53"/>
+    <mergeCell ref="A71:D71"/>
     <mergeCell ref="I9:J9"/>
     <mergeCell ref="B48:D48"/>
     <mergeCell ref="I5:J5"/>
@@ -30088,8 +30091,6 @@
     <mergeCell ref="B50:D50"/>
     <mergeCell ref="B35:D35"/>
     <mergeCell ref="B21:D21"/>
-    <mergeCell ref="A2:J2"/>
-    <mergeCell ref="C53:D53"/>
     <mergeCell ref="A78:J79"/>
     <mergeCell ref="A29:D29"/>
     <mergeCell ref="A4:J4"/>
@@ -30118,7 +30119,6 @@
     <mergeCell ref="B33:D33"/>
     <mergeCell ref="B36:D36"/>
     <mergeCell ref="C67:D67"/>
-    <mergeCell ref="A71:D71"/>
   </mergeCells>
   <conditionalFormatting sqref="B24:B25">
     <cfRule type="expression" dxfId="171" priority="13" stopIfTrue="1">

</xml_diff>

<commit_message>
Update Macro Tracker v5 workbook
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Macro_Tracker_v5.xlsx
+++ b/Macro_Tracker_v5.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/8d1bd21a83edf255/Desktop/Trading System/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="11_07BBB4D6B1A3B2E06750235655848FBF97FA3FEE" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="45" documentId="11_07BBB4D6B1A3B2E06750235655848FBF97FA3FEE" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{011C0CD2-6BF8-4F43-ABDE-ABBFBB59FF57}"/>
   <bookViews>
-    <workbookView xWindow="-38520" yWindow="-7095" windowWidth="38640" windowHeight="21120" tabRatio="500" activeTab="9" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-38520" yWindow="-7095" windowWidth="38640" windowHeight="21120" tabRatio="500" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Guide" sheetId="1" r:id="rId1"/>
@@ -5929,55 +5929,64 @@
     <xf numFmtId="0" fontId="18" fillId="0" borderId="31" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="64" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="16" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="64" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="69" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="180" fontId="71" fillId="28" borderId="31" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="29" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="182" fontId="18" fillId="29" borderId="29" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="20" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="20" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="71" fillId="28" borderId="31" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="22" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="88" fillId="0" borderId="31" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="70" fillId="30" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="181" fontId="18" fillId="29" borderId="29" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="22" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="18" fillId="29" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="69" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="74" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="18" fillId="29" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="20" fillId="29" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
+    <xf numFmtId="180" fontId="71" fillId="28" borderId="31" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="67" fillId="0" borderId="31" xfId="0" applyFont="1"/>
-    <xf numFmtId="182" fontId="18" fillId="29" borderId="29" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="71" fillId="28" borderId="31" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="181" fontId="18" fillId="29" borderId="29" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="88" fillId="0" borderId="31" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    <xf numFmtId="0" fontId="20" fillId="29" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="98" fillId="52" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="19" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="26" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="27" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="92" fillId="0" borderId="31" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="94" fillId="50" borderId="31" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="100" fillId="51" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
@@ -5985,29 +5994,20 @@
     <xf numFmtId="0" fontId="102" fillId="51" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="24" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="25" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="93" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="90" fillId="50" borderId="31" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="92" fillId="0" borderId="31" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="94" fillId="50" borderId="31" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="93" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="92" fillId="0" borderId="31" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="90" fillId="50" borderId="31" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="19" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="26" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="27" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="92" fillId="0" borderId="31" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
-    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="24" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="25" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="16" fillId="0" borderId="31" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
@@ -6047,11 +6047,11 @@
     <xf numFmtId="0" fontId="106" fillId="0" borderId="31" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
     </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="31" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="18" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="31" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -9811,11 +9811,11 @@
       </c>
     </row>
     <row r="35" spans="1:7" ht="19.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A35" s="275" t="s">
+      <c r="A35" s="276" t="s">
         <v>191</v>
       </c>
-      <c r="B35" s="276"/>
-      <c r="C35" s="276"/>
+      <c r="B35" s="277"/>
+      <c r="C35" s="277"/>
       <c r="E35" s="32" t="s">
         <v>192</v>
       </c>
@@ -9860,7 +9860,7 @@
       <c r="A38" s="39" t="s">
         <v>201</v>
       </c>
-      <c r="B38" s="277" t="s">
+      <c r="B38" s="275" t="s">
         <v>202</v>
       </c>
       <c r="C38" s="271"/>
@@ -10102,6 +10102,12 @@
     </row>
   </sheetData>
   <mergeCells count="22">
+    <mergeCell ref="B42:C42"/>
+    <mergeCell ref="A35:C35"/>
+    <mergeCell ref="B40:C40"/>
+    <mergeCell ref="E19:G19"/>
+    <mergeCell ref="A37:C37"/>
+    <mergeCell ref="B39:C39"/>
     <mergeCell ref="E4:G4"/>
     <mergeCell ref="B41:C41"/>
     <mergeCell ref="A7:C7"/>
@@ -10116,14 +10122,8 @@
     <mergeCell ref="A5:C5"/>
     <mergeCell ref="A8:C8"/>
     <mergeCell ref="A14:C14"/>
-    <mergeCell ref="B42:C42"/>
-    <mergeCell ref="A35:C35"/>
-    <mergeCell ref="B40:C40"/>
-    <mergeCell ref="E19:G19"/>
-    <mergeCell ref="A37:C37"/>
     <mergeCell ref="A18:C18"/>
     <mergeCell ref="A12:C12"/>
-    <mergeCell ref="B39:C39"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink ref="E6" location="'Bias'!A1" display="Bias  ↗" xr:uid="{00000000-0004-0000-0000-000000000000}"/>
@@ -10165,29 +10165,37 @@
     <col min="8" max="8" width="30" customWidth="1"/>
     <col min="9" max="9" width="26" customWidth="1"/>
     <col min="10" max="10" width="25.7109375" customWidth="1"/>
-    <col min="11" max="11" width="48" customWidth="1"/>
+    <col min="11" max="11" width="79.42578125" customWidth="1"/>
     <col min="12" max="12" width="3" customWidth="1"/>
-    <col min="13" max="13" width="7" customWidth="1"/>
-    <col min="14" max="15" width="11" customWidth="1"/>
-    <col min="16" max="16" width="9" customWidth="1"/>
+    <col min="13" max="13" width="23.85546875" customWidth="1"/>
+    <col min="14" max="14" width="22" customWidth="1"/>
+    <col min="15" max="15" width="27.85546875" customWidth="1"/>
+    <col min="16" max="16" width="18.140625" customWidth="1"/>
     <col min="17" max="17" width="22" customWidth="1"/>
-    <col min="18" max="18" width="9" customWidth="1"/>
-    <col min="19" max="20" width="11" customWidth="1"/>
-    <col min="21" max="21" width="12" customWidth="1"/>
-    <col min="22" max="25" width="10" customWidth="1"/>
-    <col min="26" max="28" width="9" customWidth="1"/>
-    <col min="29" max="29" width="11" customWidth="1"/>
-    <col min="30" max="30" width="10" customWidth="1"/>
-    <col min="31" max="31" width="13" customWidth="1"/>
-    <col min="32" max="32" width="10" customWidth="1"/>
-    <col min="33" max="34" width="8" customWidth="1"/>
-    <col min="35" max="35" width="7" customWidth="1"/>
-    <col min="36" max="36" width="10" customWidth="1"/>
-    <col min="37" max="37" width="12" customWidth="1"/>
-    <col min="38" max="38" width="8" customWidth="1"/>
+    <col min="18" max="18" width="18.85546875" customWidth="1"/>
+    <col min="19" max="19" width="20.42578125" customWidth="1"/>
+    <col min="20" max="20" width="22.85546875" customWidth="1"/>
+    <col min="21" max="21" width="22.42578125" customWidth="1"/>
+    <col min="22" max="22" width="17" customWidth="1"/>
+    <col min="23" max="23" width="14" customWidth="1"/>
+    <col min="24" max="24" width="15.85546875" customWidth="1"/>
+    <col min="25" max="25" width="17.7109375" customWidth="1"/>
+    <col min="26" max="26" width="13.28515625" customWidth="1"/>
+    <col min="27" max="27" width="15.7109375" customWidth="1"/>
+    <col min="28" max="28" width="15.42578125" customWidth="1"/>
+    <col min="29" max="29" width="24.42578125" customWidth="1"/>
+    <col min="30" max="30" width="14.5703125" customWidth="1"/>
+    <col min="31" max="31" width="27.85546875" customWidth="1"/>
+    <col min="32" max="32" width="12.5703125" customWidth="1"/>
+    <col min="33" max="33" width="18.85546875" customWidth="1"/>
+    <col min="34" max="34" width="15.85546875" customWidth="1"/>
+    <col min="35" max="35" width="19.140625" customWidth="1"/>
+    <col min="36" max="36" width="13.42578125" customWidth="1"/>
+    <col min="37" max="37" width="13.5703125" customWidth="1"/>
+    <col min="38" max="38" width="18.28515625" customWidth="1"/>
     <col min="39" max="39" width="26" customWidth="1"/>
     <col min="40" max="40" width="34" customWidth="1"/>
-    <col min="41" max="41" width="14" customWidth="1"/>
+    <col min="41" max="41" width="18.140625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:41" ht="33.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
@@ -10238,7 +10246,7 @@
       <c r="AN1" s="235"/>
       <c r="AO1" s="235"/>
     </row>
-    <row r="2" spans="1:41" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:41" ht="29.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="4" t="s">
         <v>3</v>
       </c>
@@ -20456,7 +20464,7 @@
       <c r="S197" s="259"/>
       <c r="T197" s="259"/>
       <c r="U197" s="261" t="str">
-        <f t="shared" ref="U197:U260" si="18">IF(OR(P197="",T197=""),"",IF(OR(AND(P197="Long",T197="LONG"),AND(P197="Short",T197="SHORT")),"WITH",IF(OR(T197="LONG",T197="SHORT"),"AGAINST","NO PERMISSION")))</f>
+        <f t="shared" ref="U197:U205" si="18">IF(OR(P197="",T197=""),"",IF(OR(AND(P197="Long",T197="LONG"),AND(P197="Short",T197="SHORT")),"WITH",IF(OR(T197="LONG",T197="SHORT"),"AGAINST","NO PERMISSION")))</f>
         <v/>
       </c>
       <c r="V197" s="259"/>
@@ -20465,7 +20473,7 @@
       <c r="Y197" s="259"/>
       <c r="Z197" s="262"/>
       <c r="AA197" s="263" t="str">
-        <f t="shared" ref="AA197:AA260" si="19">IF(OR(Z197="",$N$3=""),"",Z197/$N$3)</f>
+        <f t="shared" ref="AA197:AA205" si="19">IF(OR(Z197="",$N$3=""),"",Z197/$N$3)</f>
         <v/>
       </c>
       <c r="AB197" s="264" t="str">
@@ -20477,7 +20485,7 @@
       <c r="AE197" s="259"/>
       <c r="AF197" s="265"/>
       <c r="AG197" s="266" t="str">
-        <f t="shared" ref="AG197:AG260" si="21">IF(OR(AF197="",Z197=""),"",IFERROR(AF197/Z197,""))</f>
+        <f t="shared" ref="AG197:AG205" si="21">IF(OR(AF197="",Z197=""),"",IFERROR(AF197/Z197,""))</f>
         <v/>
       </c>
       <c r="AH197" s="261" t="str">
@@ -21455,7 +21463,7 @@
       <c r="G21" s="7"/>
       <c r="H21" s="7"/>
     </row>
-    <row r="22" spans="1:8" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:8" ht="57.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A22" s="73" t="s">
         <v>724</v>
       </c>
@@ -25102,110 +25110,110 @@
       <c r="A5" s="241">
         <v>1</v>
       </c>
-      <c r="B5" s="321" t="s">
+      <c r="B5" s="322" t="s">
         <v>929</v>
       </c>
-      <c r="C5" s="285"/>
-      <c r="D5" s="285"/>
+      <c r="C5" s="282"/>
+      <c r="D5" s="282"/>
       <c r="E5" s="280"/>
     </row>
     <row r="6" spans="1:5" ht="21" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="241">
         <v>2</v>
       </c>
-      <c r="B6" s="321" t="s">
+      <c r="B6" s="322" t="s">
         <v>930</v>
       </c>
-      <c r="C6" s="285"/>
-      <c r="D6" s="285"/>
+      <c r="C6" s="282"/>
+      <c r="D6" s="282"/>
       <c r="E6" s="280"/>
     </row>
     <row r="7" spans="1:5" ht="33.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="241">
         <v>3</v>
       </c>
-      <c r="B7" s="321" t="s">
+      <c r="B7" s="322" t="s">
         <v>931</v>
       </c>
-      <c r="C7" s="285"/>
-      <c r="D7" s="285"/>
+      <c r="C7" s="282"/>
+      <c r="D7" s="282"/>
       <c r="E7" s="280"/>
     </row>
     <row r="8" spans="1:5" ht="21" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="241">
         <v>4</v>
       </c>
-      <c r="B8" s="321" t="s">
+      <c r="B8" s="322" t="s">
         <v>932</v>
       </c>
-      <c r="C8" s="285"/>
-      <c r="D8" s="285"/>
+      <c r="C8" s="282"/>
+      <c r="D8" s="282"/>
       <c r="E8" s="280"/>
     </row>
     <row r="9" spans="1:5" ht="21" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="241">
         <v>5</v>
       </c>
-      <c r="B9" s="321" t="s">
+      <c r="B9" s="322" t="s">
         <v>933</v>
       </c>
-      <c r="C9" s="285"/>
-      <c r="D9" s="285"/>
+      <c r="C9" s="282"/>
+      <c r="D9" s="282"/>
       <c r="E9" s="280"/>
     </row>
     <row r="10" spans="1:5" ht="21" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="241">
         <v>6</v>
       </c>
-      <c r="B10" s="321" t="s">
+      <c r="B10" s="322" t="s">
         <v>934</v>
       </c>
-      <c r="C10" s="285"/>
-      <c r="D10" s="285"/>
+      <c r="C10" s="282"/>
+      <c r="D10" s="282"/>
       <c r="E10" s="280"/>
     </row>
     <row r="11" spans="1:5" ht="21" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="241">
         <v>7</v>
       </c>
-      <c r="B11" s="321" t="s">
+      <c r="B11" s="322" t="s">
         <v>935</v>
       </c>
-      <c r="C11" s="285"/>
-      <c r="D11" s="285"/>
+      <c r="C11" s="282"/>
+      <c r="D11" s="282"/>
       <c r="E11" s="280"/>
     </row>
     <row r="12" spans="1:5" ht="21" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="241">
         <v>8</v>
       </c>
-      <c r="B12" s="321" t="s">
+      <c r="B12" s="322" t="s">
         <v>936</v>
       </c>
-      <c r="C12" s="285"/>
-      <c r="D12" s="285"/>
+      <c r="C12" s="282"/>
+      <c r="D12" s="282"/>
       <c r="E12" s="280"/>
     </row>
     <row r="13" spans="1:5" ht="21" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="241">
         <v>9</v>
       </c>
-      <c r="B13" s="321" t="s">
+      <c r="B13" s="322" t="s">
         <v>937</v>
       </c>
-      <c r="C13" s="285"/>
-      <c r="D13" s="285"/>
+      <c r="C13" s="282"/>
+      <c r="D13" s="282"/>
       <c r="E13" s="280"/>
     </row>
     <row r="14" spans="1:5" ht="21" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="241">
         <v>10</v>
       </c>
-      <c r="B14" s="321" t="s">
+      <c r="B14" s="322" t="s">
         <v>938</v>
       </c>
-      <c r="C14" s="285"/>
-      <c r="D14" s="285"/>
+      <c r="C14" s="282"/>
+      <c r="D14" s="282"/>
       <c r="E14" s="280"/>
     </row>
     <row r="16" spans="1:5" ht="26.1" customHeight="1" x14ac:dyDescent="0.25">
@@ -25414,7 +25422,7 @@
       <c r="E29" s="269"/>
     </row>
     <row r="30" spans="1:5" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B30" s="322" t="s">
+      <c r="B30" s="321" t="s">
         <v>995</v>
       </c>
       <c r="C30" s="273"/>
@@ -25422,7 +25430,7 @@
       <c r="E30" s="273"/>
     </row>
     <row r="31" spans="1:5" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B31" s="322" t="s">
+      <c r="B31" s="321" t="s">
         <v>996</v>
       </c>
       <c r="C31" s="273"/>
@@ -25430,7 +25438,7 @@
       <c r="E31" s="273"/>
     </row>
     <row r="32" spans="1:5" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B32" s="322" t="s">
+      <c r="B32" s="321" t="s">
         <v>997</v>
       </c>
       <c r="C32" s="273"/>
@@ -25438,7 +25446,7 @@
       <c r="E32" s="273"/>
     </row>
     <row r="33" spans="2:5" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B33" s="322" t="s">
+      <c r="B33" s="321" t="s">
         <v>998</v>
       </c>
       <c r="C33" s="273"/>
@@ -25446,7 +25454,7 @@
       <c r="E33" s="273"/>
     </row>
     <row r="34" spans="2:5" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B34" s="322" t="s">
+      <c r="B34" s="321" t="s">
         <v>999</v>
       </c>
       <c r="C34" s="273"/>
@@ -25455,6 +25463,9 @@
     </row>
   </sheetData>
   <mergeCells count="19">
+    <mergeCell ref="A16:E16"/>
+    <mergeCell ref="B7:E7"/>
+    <mergeCell ref="B31:E31"/>
     <mergeCell ref="B34:E34"/>
     <mergeCell ref="B10:E10"/>
     <mergeCell ref="A2:E2"/>
@@ -25471,9 +25482,6 @@
     <mergeCell ref="B33:E33"/>
     <mergeCell ref="B5:E5"/>
     <mergeCell ref="B32:E32"/>
-    <mergeCell ref="A16:E16"/>
-    <mergeCell ref="B7:E7"/>
-    <mergeCell ref="B31:E31"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink ref="E1" location="'Guide'!A1" display="← Guide" xr:uid="{00000000-0004-0000-0D00-000000000000}"/>
@@ -25550,7 +25558,7 @@
     </row>
     <row r="3" spans="1:33" ht="8.1" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="4" spans="1:33" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="287" t="s">
+      <c r="A4" s="278" t="s">
         <v>255</v>
       </c>
       <c r="B4" s="269"/>
@@ -25568,9 +25576,9 @@
       <c r="A5" s="281" t="s">
         <v>246</v>
       </c>
-      <c r="B5" s="285"/>
+      <c r="B5" s="282"/>
       <c r="C5" s="280"/>
-      <c r="D5" s="292">
+      <c r="D5" s="279">
         <f ca="1">TODAY()</f>
         <v>46310</v>
       </c>
@@ -25579,11 +25587,11 @@
         <v>256</v>
       </c>
       <c r="G5" s="280"/>
-      <c r="H5" s="283">
+      <c r="H5" s="284">
         <v>0</v>
       </c>
       <c r="I5" s="280"/>
-      <c r="J5" s="279" t="str">
+      <c r="J5" s="293" t="str">
         <f ca="1">COUNTIFS(Events!$A$5:$A$304,TODAY(),Events!$K$5:$K$304,"&gt;="&amp;$AC$5)&amp;" event(s) today"</f>
         <v>11 event(s) today</v>
       </c>
@@ -25597,9 +25605,9 @@
       <c r="A6" s="281" t="s">
         <v>257</v>
       </c>
-      <c r="B6" s="285"/>
+      <c r="B6" s="282"/>
       <c r="C6" s="280"/>
-      <c r="D6" s="283" t="s">
+      <c r="D6" s="284" t="s">
         <v>258</v>
       </c>
       <c r="E6" s="280"/>
@@ -25607,34 +25615,34 @@
         <v>259</v>
       </c>
       <c r="G6" s="280"/>
-      <c r="H6" s="284">
+      <c r="H6" s="292">
         <f ca="1">TODAY()-WEEKDAY(TODAY(),3)+IF(WEEKDAY(TODAY(),2)&gt;5,7,0)+7*$H$5</f>
         <v>46307</v>
       </c>
       <c r="I6" s="280"/>
-      <c r="J6" s="286"/>
+      <c r="J6" s="287"/>
       <c r="K6" s="280"/>
     </row>
     <row r="7" spans="1:33" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="281" t="s">
         <v>260</v>
       </c>
-      <c r="B7" s="285"/>
+      <c r="B7" s="282"/>
       <c r="C7" s="280"/>
-      <c r="D7" s="290" t="str">
+      <c r="D7" s="288" t="str">
         <f ca="1">IFERROR(INDEX(Events!$C$5:$C$304,MATCH(_xlfn.MINIFS(Events!$L$5:$L$304,Events!$D$5:$D$304,"High",Events!$L$5:$L$304,"&gt;="&amp;NOW()),Events!$L$5:$L$304,0))&amp;"  "&amp;INDEX(Events!$F$5:$F$304,MATCH(_xlfn.MINIFS(Events!$L$5:$L$304,Events!$D$5:$D$304,"High",Events!$L$5:$L$304,"&gt;="&amp;NOW()),Events!$L$5:$L$304,0))&amp;"  —  "&amp;TEXT(_xlfn.MINIFS(Events!$L$5:$L$304,Events!$D$5:$D$304,"High",Events!$L$5:$L$304,"&gt;="&amp;NOW()),"ddd d mmm hh:mm")&amp;"  (in "&amp;INT(_xlfn.MINIFS(Events!$L$5:$L$304,Events!$D$5:$D$304,"High",Events!$L$5:$L$304,"&gt;="&amp;NOW()))-TODAY()&amp;" days)","none scheduled")</f>
         <v>USD  Core PPI m/m  —  Thu 15 Oct 14:30  (in 0 days)</v>
       </c>
-      <c r="E7" s="285"/>
-      <c r="F7" s="285"/>
-      <c r="G7" s="285"/>
-      <c r="H7" s="285"/>
-      <c r="I7" s="285"/>
-      <c r="J7" s="285"/>
+      <c r="E7" s="282"/>
+      <c r="F7" s="282"/>
+      <c r="G7" s="282"/>
+      <c r="H7" s="282"/>
+      <c r="I7" s="282"/>
+      <c r="J7" s="282"/>
       <c r="K7" s="280"/>
     </row>
     <row r="9" spans="1:33" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="287" t="s">
+      <c r="A9" s="278" t="s">
         <v>261</v>
       </c>
       <c r="B9" s="269"/>
@@ -25647,7 +25655,7 @@
       <c r="I9" s="269"/>
       <c r="J9" s="269"/>
       <c r="K9" s="269"/>
-      <c r="M9" s="287" t="s">
+      <c r="M9" s="278" t="s">
         <v>262</v>
       </c>
       <c r="N9" s="269"/>
@@ -25669,32 +25677,32 @@
       <c r="A10" s="143" t="s">
         <v>263</v>
       </c>
-      <c r="B10" s="278">
+      <c r="B10" s="289">
         <f ca="1">$H$6+0</f>
         <v>46307</v>
       </c>
       <c r="C10" s="273"/>
-      <c r="D10" s="278">
+      <c r="D10" s="289">
         <f ca="1">$H$6+1</f>
         <v>46308</v>
       </c>
       <c r="E10" s="273"/>
-      <c r="F10" s="278">
+      <c r="F10" s="289">
         <f ca="1">$H$6+2</f>
         <v>46309</v>
       </c>
       <c r="G10" s="273"/>
-      <c r="H10" s="278">
+      <c r="H10" s="289">
         <f ca="1">$H$6+3</f>
         <v>46310</v>
       </c>
       <c r="I10" s="273"/>
-      <c r="J10" s="278">
+      <c r="J10" s="289">
         <f ca="1">$H$6+4</f>
         <v>46311</v>
       </c>
       <c r="K10" s="273"/>
-      <c r="M10" s="282" t="str">
+      <c r="M10" s="291" t="str">
         <f ca="1">TEXT(DATE(YEAR($H$6),MONTH($H$6),1),"mmmm yyyy")</f>
         <v>October 2026</v>
       </c>
@@ -25704,7 +25712,7 @@
       <c r="Q10" s="273"/>
       <c r="R10" s="273"/>
       <c r="S10" s="273"/>
-      <c r="U10" s="282" t="str">
+      <c r="U10" s="291" t="str">
         <f ca="1">TEXT(EDATE(DATE(YEAR($H$6),MONTH($H$6),1),1),"mmmm yyyy")</f>
         <v>November 2026</v>
       </c>
@@ -26657,7 +26665,7 @@
         <f ca="1">IF($AG19="","",IF(INDEX(Events!$D$5:$D$304,$AG19)="High","●  ",IF(INDEX(Events!$D$5:$D$304,$AG19)="Medium","○  ","    "))&amp;IF(INDEX(Events!$B$5:$B$304,$AG19)="","all day",TEXT(INDEX(Events!$B$5:$B$304,$AG19),"hh:mm"))&amp;"   "&amp;INDEX(Events!$C$5:$C$304,$AG19)&amp;"   "&amp;INDEX(Events!$F$5:$F$304,$AG19))</f>
         <v/>
       </c>
-      <c r="M19" s="282" t="str">
+      <c r="M19" s="291" t="str">
         <f ca="1">TEXT(EDATE(DATE(YEAR($H$6),MONTH($H$6),1),2),"mmmm yyyy")</f>
         <v>December 2026</v>
       </c>
@@ -26667,7 +26675,7 @@
       <c r="Q19" s="273"/>
       <c r="R19" s="273"/>
       <c r="S19" s="273"/>
-      <c r="U19" s="282" t="str">
+      <c r="U19" s="291" t="str">
         <f ca="1">TEXT(EDATE(DATE(YEAR($H$6),MONTH($H$6),1),3),"mmmm yyyy")</f>
         <v>January 2027</v>
       </c>
@@ -27048,7 +27056,7 @@
       </c>
     </row>
     <row r="23" spans="1:33" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B23" s="291" t="s">
+      <c r="B23" s="290" t="s">
         <v>271</v>
       </c>
       <c r="C23" s="273"/>
@@ -27176,7 +27184,7 @@
       </c>
     </row>
     <row r="25" spans="1:33" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A25" s="287" t="s">
+      <c r="A25" s="278" t="s">
         <v>272</v>
       </c>
       <c r="B25" s="269"/>
@@ -27247,18 +27255,18 @@
       </c>
     </row>
     <row r="26" spans="1:33" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B26" s="288" t="s">
+      <c r="B26" s="285" t="s">
         <v>273</v>
       </c>
-      <c r="C26" s="289"/>
-      <c r="D26" s="288" t="s">
+      <c r="C26" s="286"/>
+      <c r="D26" s="285" t="s">
         <v>274</v>
       </c>
-      <c r="E26" s="289"/>
-      <c r="F26" s="288" t="s">
+      <c r="E26" s="286"/>
+      <c r="F26" s="285" t="s">
         <v>275</v>
       </c>
-      <c r="G26" s="289"/>
+      <c r="G26" s="286"/>
       <c r="M26" s="148">
         <f ca="1">(EDATE(DATE(YEAR($H$6),MONTH($H$6),1),2)-WEEKDAY(EDATE(DATE(YEAR($H$6),MONTH($H$6),1),2),3))+35</f>
         <v>46391</v>
@@ -27335,7 +27343,7 @@
       <c r="G27" s="146" t="s">
         <v>281</v>
       </c>
-      <c r="M27" s="293" t="s">
+      <c r="M27" s="283" t="s">
         <v>282</v>
       </c>
       <c r="N27" s="273"/>
@@ -27529,6 +27537,20 @@
     </row>
   </sheetData>
   <mergeCells count="30">
+    <mergeCell ref="J5:K5"/>
+    <mergeCell ref="F10:G10"/>
+    <mergeCell ref="H10:I10"/>
+    <mergeCell ref="J10:K10"/>
+    <mergeCell ref="F6:G6"/>
+    <mergeCell ref="B10:C10"/>
+    <mergeCell ref="B23:K23"/>
+    <mergeCell ref="U19:AA19"/>
+    <mergeCell ref="D6:E6"/>
+    <mergeCell ref="U10:AA10"/>
+    <mergeCell ref="M19:S19"/>
+    <mergeCell ref="H6:I6"/>
+    <mergeCell ref="M10:S10"/>
+    <mergeCell ref="D10:E10"/>
     <mergeCell ref="A4:K4"/>
     <mergeCell ref="D5:E5"/>
     <mergeCell ref="A6:C6"/>
@@ -27545,20 +27567,6 @@
     <mergeCell ref="A25:K25"/>
     <mergeCell ref="F26:G26"/>
     <mergeCell ref="D7:K7"/>
-    <mergeCell ref="B10:C10"/>
-    <mergeCell ref="B23:K23"/>
-    <mergeCell ref="U19:AA19"/>
-    <mergeCell ref="D6:E6"/>
-    <mergeCell ref="U10:AA10"/>
-    <mergeCell ref="M19:S19"/>
-    <mergeCell ref="H6:I6"/>
-    <mergeCell ref="M10:S10"/>
-    <mergeCell ref="D10:E10"/>
-    <mergeCell ref="J5:K5"/>
-    <mergeCell ref="F10:G10"/>
-    <mergeCell ref="H10:I10"/>
-    <mergeCell ref="J10:K10"/>
-    <mergeCell ref="F6:G6"/>
   </mergeCells>
   <conditionalFormatting sqref="B10">
     <cfRule type="expression" dxfId="253" priority="19" stopIfTrue="1">
@@ -28493,7 +28501,7 @@
       </c>
     </row>
     <row r="2" spans="1:10" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="307" t="s">
+      <c r="A2" s="298" t="s">
         <v>354</v>
       </c>
       <c r="B2" s="273"/>
@@ -28508,7 +28516,7 @@
     </row>
     <row r="3" spans="1:10" ht="8.1" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="4" spans="1:10" ht="26.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="301" t="s">
+      <c r="A4" s="302" t="s">
         <v>355</v>
       </c>
       <c r="B4" s="269"/>
@@ -28544,7 +28552,7 @@
       <c r="H5" s="184" t="s">
         <v>360</v>
       </c>
-      <c r="I5" s="300" t="s">
+      <c r="I5" s="299" t="s">
         <v>361</v>
       </c>
       <c r="J5" s="273"/>
@@ -28574,7 +28582,7 @@
         <f>IF(TRIM(F6)="","User: —",IF(AND(UPPER(TRIM(B6))=UPPER(TRIM(C6)),UPPER(TRIM(C6))=UPPER(TRIM(F6))),"ALL AGREE",IF(OR(UPPER(TRIM(B6))=UPPER(TRIM(C6)),UPPER(TRIM(C6))=UPPER(TRIM(F6)),UPPER(TRIM(B6))=UPPER(TRIM(F6))),"2 OF 3","SPLIT")))</f>
         <v>2 OF 3</v>
       </c>
-      <c r="I6" s="295" t="str">
+      <c r="I6" s="300" t="str">
         <f ca="1">IFERROR(IF(MIN(IF(_xlfn.MINIFS(Events!$L$5:$L$304,Events!$C$5:$C$304,"EUR",Events!$D$5:$D$304,"High",Events!$L$5:$L$304,"&gt;="&amp;NOW())=0,9000000000,_xlfn.MINIFS(Events!$L$5:$L$304,Events!$C$5:$C$304,"EUR",Events!$D$5:$D$304,"High",Events!$L$5:$L$304,"&gt;="&amp;NOW())),IF(_xlfn.MINIFS(Events!$L$5:$L$304,Events!$C$5:$C$304,"USD",Events!$D$5:$D$304,"High",Events!$L$5:$L$304,"&gt;="&amp;NOW())=0,9000000000,_xlfn.MINIFS(Events!$L$5:$L$304,Events!$C$5:$C$304,"USD",Events!$D$5:$D$304,"High",Events!$L$5:$L$304,"&gt;="&amp;NOW())))&gt;900000000,"none scheduled",TEXT(MIN(IF(_xlfn.MINIFS(Events!$L$5:$L$304,Events!$C$5:$C$304,"EUR",Events!$D$5:$D$304,"High",Events!$L$5:$L$304,"&gt;="&amp;NOW())=0,9000000000,_xlfn.MINIFS(Events!$L$5:$L$304,Events!$C$5:$C$304,"EUR",Events!$D$5:$D$304,"High",Events!$L$5:$L$304,"&gt;="&amp;NOW())),IF(_xlfn.MINIFS(Events!$L$5:$L$304,Events!$C$5:$C$304,"USD",Events!$D$5:$D$304,"High",Events!$L$5:$L$304,"&gt;="&amp;NOW())=0,9000000000,_xlfn.MINIFS(Events!$L$5:$L$304,Events!$C$5:$C$304,"USD",Events!$D$5:$D$304,"High",Events!$L$5:$L$304,"&gt;="&amp;NOW()))),"ddd d mmm")&amp;"  "&amp;INDEX(Events!$C$5:$C$304,MATCH(MIN(IF(_xlfn.MINIFS(Events!$L$5:$L$304,Events!$C$5:$C$304,"EUR",Events!$D$5:$D$304,"High",Events!$L$5:$L$304,"&gt;="&amp;NOW())=0,9000000000,_xlfn.MINIFS(Events!$L$5:$L$304,Events!$C$5:$C$304,"EUR",Events!$D$5:$D$304,"High",Events!$L$5:$L$304,"&gt;="&amp;NOW())),IF(_xlfn.MINIFS(Events!$L$5:$L$304,Events!$C$5:$C$304,"USD",Events!$D$5:$D$304,"High",Events!$L$5:$L$304,"&gt;="&amp;NOW())=0,9000000000,_xlfn.MINIFS(Events!$L$5:$L$304,Events!$C$5:$C$304,"USD",Events!$D$5:$D$304,"High",Events!$L$5:$L$304,"&gt;="&amp;NOW()))),Events!$L$5:$L$304,0))&amp;"  "&amp;INDEX(Events!$F$5:$F$304,MATCH(MIN(IF(_xlfn.MINIFS(Events!$L$5:$L$304,Events!$C$5:$C$304,"EUR",Events!$D$5:$D$304,"High",Events!$L$5:$L$304,"&gt;="&amp;NOW())=0,9000000000,_xlfn.MINIFS(Events!$L$5:$L$304,Events!$C$5:$C$304,"EUR",Events!$D$5:$D$304,"High",Events!$L$5:$L$304,"&gt;="&amp;NOW())),IF(_xlfn.MINIFS(Events!$L$5:$L$304,Events!$C$5:$C$304,"USD",Events!$D$5:$D$304,"High",Events!$L$5:$L$304,"&gt;="&amp;NOW())=0,9000000000,_xlfn.MINIFS(Events!$L$5:$L$304,Events!$C$5:$C$304,"USD",Events!$D$5:$D$304,"High",Events!$L$5:$L$304,"&gt;="&amp;NOW()))),Events!$L$5:$L$304,0))),"none scheduled")</f>
         <v>Thu 15 Oct  USD  Core PPI m/m</v>
       </c>
@@ -28605,7 +28613,7 @@
         <f>IF(TRIM(F7)="","User: —",IF(AND(UPPER(TRIM(B7))=UPPER(TRIM(C7)),UPPER(TRIM(C7))=UPPER(TRIM(F7))),"ALL AGREE",IF(OR(UPPER(TRIM(B7))=UPPER(TRIM(C7)),UPPER(TRIM(C7))=UPPER(TRIM(F7)),UPPER(TRIM(B7))=UPPER(TRIM(F7))),"2 OF 3","SPLIT")))</f>
         <v>ALL AGREE</v>
       </c>
-      <c r="I7" s="295" t="str">
+      <c r="I7" s="300" t="str">
         <f ca="1">IFERROR(IF(MIN(IF(_xlfn.MINIFS(Events!$L$5:$L$304,Events!$C$5:$C$304,"GBP",Events!$D$5:$D$304,"High",Events!$L$5:$L$304,"&gt;="&amp;NOW())=0,9000000000,_xlfn.MINIFS(Events!$L$5:$L$304,Events!$C$5:$C$304,"GBP",Events!$D$5:$D$304,"High",Events!$L$5:$L$304,"&gt;="&amp;NOW())),IF(_xlfn.MINIFS(Events!$L$5:$L$304,Events!$C$5:$C$304,"USD",Events!$D$5:$D$304,"High",Events!$L$5:$L$304,"&gt;="&amp;NOW())=0,9000000000,_xlfn.MINIFS(Events!$L$5:$L$304,Events!$C$5:$C$304,"USD",Events!$D$5:$D$304,"High",Events!$L$5:$L$304,"&gt;="&amp;NOW())))&gt;900000000,"none scheduled",TEXT(MIN(IF(_xlfn.MINIFS(Events!$L$5:$L$304,Events!$C$5:$C$304,"GBP",Events!$D$5:$D$304,"High",Events!$L$5:$L$304,"&gt;="&amp;NOW())=0,9000000000,_xlfn.MINIFS(Events!$L$5:$L$304,Events!$C$5:$C$304,"GBP",Events!$D$5:$D$304,"High",Events!$L$5:$L$304,"&gt;="&amp;NOW())),IF(_xlfn.MINIFS(Events!$L$5:$L$304,Events!$C$5:$C$304,"USD",Events!$D$5:$D$304,"High",Events!$L$5:$L$304,"&gt;="&amp;NOW())=0,9000000000,_xlfn.MINIFS(Events!$L$5:$L$304,Events!$C$5:$C$304,"USD",Events!$D$5:$D$304,"High",Events!$L$5:$L$304,"&gt;="&amp;NOW()))),"ddd d mmm")&amp;"  "&amp;INDEX(Events!$C$5:$C$304,MATCH(MIN(IF(_xlfn.MINIFS(Events!$L$5:$L$304,Events!$C$5:$C$304,"GBP",Events!$D$5:$D$304,"High",Events!$L$5:$L$304,"&gt;="&amp;NOW())=0,9000000000,_xlfn.MINIFS(Events!$L$5:$L$304,Events!$C$5:$C$304,"GBP",Events!$D$5:$D$304,"High",Events!$L$5:$L$304,"&gt;="&amp;NOW())),IF(_xlfn.MINIFS(Events!$L$5:$L$304,Events!$C$5:$C$304,"USD",Events!$D$5:$D$304,"High",Events!$L$5:$L$304,"&gt;="&amp;NOW())=0,9000000000,_xlfn.MINIFS(Events!$L$5:$L$304,Events!$C$5:$C$304,"USD",Events!$D$5:$D$304,"High",Events!$L$5:$L$304,"&gt;="&amp;NOW()))),Events!$L$5:$L$304,0))&amp;"  "&amp;INDEX(Events!$F$5:$F$304,MATCH(MIN(IF(_xlfn.MINIFS(Events!$L$5:$L$304,Events!$C$5:$C$304,"GBP",Events!$D$5:$D$304,"High",Events!$L$5:$L$304,"&gt;="&amp;NOW())=0,9000000000,_xlfn.MINIFS(Events!$L$5:$L$304,Events!$C$5:$C$304,"GBP",Events!$D$5:$D$304,"High",Events!$L$5:$L$304,"&gt;="&amp;NOW())),IF(_xlfn.MINIFS(Events!$L$5:$L$304,Events!$C$5:$C$304,"USD",Events!$D$5:$D$304,"High",Events!$L$5:$L$304,"&gt;="&amp;NOW())=0,9000000000,_xlfn.MINIFS(Events!$L$5:$L$304,Events!$C$5:$C$304,"USD",Events!$D$5:$D$304,"High",Events!$L$5:$L$304,"&gt;="&amp;NOW()))),Events!$L$5:$L$304,0))),"none scheduled")</f>
         <v>Thu 15 Oct  USD  Core PPI m/m</v>
       </c>
@@ -28636,7 +28644,7 @@
         <f>IF(TRIM(F8)="","User: —",IF(AND(UPPER(TRIM(B8))=UPPER(TRIM(C8)),UPPER(TRIM(C8))=UPPER(TRIM(F8))),"ALL AGREE",IF(OR(UPPER(TRIM(B8))=UPPER(TRIM(C8)),UPPER(TRIM(C8))=UPPER(TRIM(F8)),UPPER(TRIM(B8))=UPPER(TRIM(F8))),"2 OF 3","SPLIT")))</f>
         <v>2 OF 3</v>
       </c>
-      <c r="I8" s="295" t="str">
+      <c r="I8" s="300" t="str">
         <f ca="1">IFERROR(IF(MIN(IF(_xlfn.MINIFS(Events!$L$5:$L$304,Events!$C$5:$C$304,"USD",Events!$D$5:$D$304,"High",Events!$L$5:$L$304,"&gt;="&amp;NOW())=0,9000000000,_xlfn.MINIFS(Events!$L$5:$L$304,Events!$C$5:$C$304,"USD",Events!$D$5:$D$304,"High",Events!$L$5:$L$304,"&gt;="&amp;NOW())),IF(_xlfn.MINIFS(Events!$L$5:$L$304,Events!$C$5:$C$304,"JPY",Events!$D$5:$D$304,"High",Events!$L$5:$L$304,"&gt;="&amp;NOW())=0,9000000000,_xlfn.MINIFS(Events!$L$5:$L$304,Events!$C$5:$C$304,"JPY",Events!$D$5:$D$304,"High",Events!$L$5:$L$304,"&gt;="&amp;NOW())))&gt;900000000,"none scheduled",TEXT(MIN(IF(_xlfn.MINIFS(Events!$L$5:$L$304,Events!$C$5:$C$304,"USD",Events!$D$5:$D$304,"High",Events!$L$5:$L$304,"&gt;="&amp;NOW())=0,9000000000,_xlfn.MINIFS(Events!$L$5:$L$304,Events!$C$5:$C$304,"USD",Events!$D$5:$D$304,"High",Events!$L$5:$L$304,"&gt;="&amp;NOW())),IF(_xlfn.MINIFS(Events!$L$5:$L$304,Events!$C$5:$C$304,"JPY",Events!$D$5:$D$304,"High",Events!$L$5:$L$304,"&gt;="&amp;NOW())=0,9000000000,_xlfn.MINIFS(Events!$L$5:$L$304,Events!$C$5:$C$304,"JPY",Events!$D$5:$D$304,"High",Events!$L$5:$L$304,"&gt;="&amp;NOW()))),"ddd d mmm")&amp;"  "&amp;INDEX(Events!$C$5:$C$304,MATCH(MIN(IF(_xlfn.MINIFS(Events!$L$5:$L$304,Events!$C$5:$C$304,"USD",Events!$D$5:$D$304,"High",Events!$L$5:$L$304,"&gt;="&amp;NOW())=0,9000000000,_xlfn.MINIFS(Events!$L$5:$L$304,Events!$C$5:$C$304,"USD",Events!$D$5:$D$304,"High",Events!$L$5:$L$304,"&gt;="&amp;NOW())),IF(_xlfn.MINIFS(Events!$L$5:$L$304,Events!$C$5:$C$304,"JPY",Events!$D$5:$D$304,"High",Events!$L$5:$L$304,"&gt;="&amp;NOW())=0,9000000000,_xlfn.MINIFS(Events!$L$5:$L$304,Events!$C$5:$C$304,"JPY",Events!$D$5:$D$304,"High",Events!$L$5:$L$304,"&gt;="&amp;NOW()))),Events!$L$5:$L$304,0))&amp;"  "&amp;INDEX(Events!$F$5:$F$304,MATCH(MIN(IF(_xlfn.MINIFS(Events!$L$5:$L$304,Events!$C$5:$C$304,"USD",Events!$D$5:$D$304,"High",Events!$L$5:$L$304,"&gt;="&amp;NOW())=0,9000000000,_xlfn.MINIFS(Events!$L$5:$L$304,Events!$C$5:$C$304,"USD",Events!$D$5:$D$304,"High",Events!$L$5:$L$304,"&gt;="&amp;NOW())),IF(_xlfn.MINIFS(Events!$L$5:$L$304,Events!$C$5:$C$304,"JPY",Events!$D$5:$D$304,"High",Events!$L$5:$L$304,"&gt;="&amp;NOW())=0,9000000000,_xlfn.MINIFS(Events!$L$5:$L$304,Events!$C$5:$C$304,"JPY",Events!$D$5:$D$304,"High",Events!$L$5:$L$304,"&gt;="&amp;NOW()))),Events!$L$5:$L$304,0))),"none scheduled")</f>
         <v>Thu 15 Oct  USD  Core PPI m/m</v>
       </c>
@@ -28667,14 +28675,14 @@
         <f>IF(TRIM(F9)="","User: —",IF(AND(UPPER(TRIM(B9))=UPPER(TRIM(C9)),UPPER(TRIM(C9))=UPPER(TRIM(F9))),"ALL AGREE",IF(OR(UPPER(TRIM(B9))=UPPER(TRIM(C9)),UPPER(TRIM(C9))=UPPER(TRIM(F9)),UPPER(TRIM(B9))=UPPER(TRIM(F9))),"2 OF 3","SPLIT")))</f>
         <v>ALL AGREE</v>
       </c>
-      <c r="I9" s="295" t="str">
+      <c r="I9" s="300" t="str">
         <f ca="1">IFERROR(IF(MIN(IF(_xlfn.MINIFS(Events!$L$5:$L$304,Events!$C$5:$C$304,"USD",Events!$D$5:$D$304,"High",Events!$L$5:$L$304,"&gt;="&amp;NOW())=0,9000000000,_xlfn.MINIFS(Events!$L$5:$L$304,Events!$C$5:$C$304,"USD",Events!$D$5:$D$304,"High",Events!$L$5:$L$304,"&gt;="&amp;NOW())))&gt;900000000,"none scheduled",TEXT(MIN(IF(_xlfn.MINIFS(Events!$L$5:$L$304,Events!$C$5:$C$304,"USD",Events!$D$5:$D$304,"High",Events!$L$5:$L$304,"&gt;="&amp;NOW())=0,9000000000,_xlfn.MINIFS(Events!$L$5:$L$304,Events!$C$5:$C$304,"USD",Events!$D$5:$D$304,"High",Events!$L$5:$L$304,"&gt;="&amp;NOW()))),"ddd d mmm")&amp;"  "&amp;INDEX(Events!$C$5:$C$304,MATCH(MIN(IF(_xlfn.MINIFS(Events!$L$5:$L$304,Events!$C$5:$C$304,"USD",Events!$D$5:$D$304,"High",Events!$L$5:$L$304,"&gt;="&amp;NOW())=0,9000000000,_xlfn.MINIFS(Events!$L$5:$L$304,Events!$C$5:$C$304,"USD",Events!$D$5:$D$304,"High",Events!$L$5:$L$304,"&gt;="&amp;NOW()))),Events!$L$5:$L$304,0))&amp;"  "&amp;INDEX(Events!$F$5:$F$304,MATCH(MIN(IF(_xlfn.MINIFS(Events!$L$5:$L$304,Events!$C$5:$C$304,"USD",Events!$D$5:$D$304,"High",Events!$L$5:$L$304,"&gt;="&amp;NOW())=0,9000000000,_xlfn.MINIFS(Events!$L$5:$L$304,Events!$C$5:$C$304,"USD",Events!$D$5:$D$304,"High",Events!$L$5:$L$304,"&gt;="&amp;NOW()))),Events!$L$5:$L$304,0))),"none scheduled")</f>
         <v>Thu 15 Oct  USD  Core PPI m/m</v>
       </c>
       <c r="J9" s="280"/>
     </row>
     <row r="10" spans="1:10" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="302" t="s">
+      <c r="A10" s="305" t="s">
         <v>367</v>
       </c>
       <c r="B10" s="273"/>
@@ -28688,7 +28696,7 @@
       <c r="J10" s="273"/>
     </row>
     <row r="12" spans="1:10" ht="26.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="301" t="s">
+      <c r="A12" s="302" t="s">
         <v>368</v>
       </c>
       <c r="B12" s="269"/>
@@ -28716,7 +28724,7 @@
       <c r="J14" s="193"/>
     </row>
     <row r="15" spans="1:10" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="300" t="s">
+      <c r="A15" s="299" t="s">
         <v>370</v>
       </c>
       <c r="B15" s="273"/>
@@ -28745,7 +28753,7 @@
       <c r="B16" s="294" t="s">
         <v>376</v>
       </c>
-      <c r="C16" s="285"/>
+      <c r="C16" s="282"/>
       <c r="D16" s="280"/>
       <c r="F16" s="195" t="s">
         <v>377</v>
@@ -28770,7 +28778,7 @@
       <c r="B17" s="294" t="s">
         <v>379</v>
       </c>
-      <c r="C17" s="285"/>
+      <c r="C17" s="282"/>
       <c r="D17" s="280"/>
       <c r="F17" s="195" t="s">
         <v>380</v>
@@ -28799,7 +28807,7 @@
       <c r="B18" s="294" t="s">
         <v>382</v>
       </c>
-      <c r="C18" s="285"/>
+      <c r="C18" s="282"/>
       <c r="D18" s="280"/>
       <c r="F18" s="195" t="s">
         <v>383</v>
@@ -28820,11 +28828,11 @@
       <c r="A19" s="194" t="s">
         <v>384</v>
       </c>
-      <c r="B19" s="296" t="str">
+      <c r="B19" s="301" t="str">
         <f ca="1">IF(Scorecard!D5="","not in Events list",TEXT(Scorecard!D5,"ddd d mmm yyyy")&amp;"  —  in "&amp;(Scorecard!D5-TODAY())&amp;" days")</f>
         <v>Wed 28 Oct 2026  —  in 13 days</v>
       </c>
-      <c r="C19" s="285"/>
+      <c r="C19" s="282"/>
       <c r="D19" s="280"/>
       <c r="F19" s="195" t="s">
         <v>385</v>
@@ -28853,7 +28861,7 @@
       <c r="B20" s="294" t="s">
         <v>387</v>
       </c>
-      <c r="C20" s="285"/>
+      <c r="C20" s="282"/>
       <c r="D20" s="280"/>
       <c r="F20" s="195" t="s">
         <v>388</v>
@@ -28877,7 +28885,7 @@
       <c r="B21" s="294" t="s">
         <v>390</v>
       </c>
-      <c r="C21" s="285"/>
+      <c r="C21" s="282"/>
       <c r="D21" s="280"/>
       <c r="F21" s="195" t="s">
         <v>391</v>
@@ -28901,7 +28909,7 @@
       <c r="B22" s="294" t="s">
         <v>393</v>
       </c>
-      <c r="C22" s="285"/>
+      <c r="C22" s="282"/>
       <c r="D22" s="280"/>
       <c r="F22" s="195" t="s">
         <v>394</v>
@@ -28924,7 +28932,7 @@
       <c r="B23" s="294" t="s">
         <v>396</v>
       </c>
-      <c r="C23" s="285"/>
+      <c r="C23" s="282"/>
       <c r="D23" s="280"/>
       <c r="F23" s="195" t="s">
         <v>397</v>
@@ -29012,7 +29020,7 @@
       <c r="J28" s="206"/>
     </row>
     <row r="29" spans="1:10" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A29" s="300" t="s">
+      <c r="A29" s="299" t="s">
         <v>370</v>
       </c>
       <c r="B29" s="273"/>
@@ -29041,7 +29049,7 @@
       <c r="B30" s="294" t="s">
         <v>405</v>
       </c>
-      <c r="C30" s="285"/>
+      <c r="C30" s="282"/>
       <c r="D30" s="280"/>
       <c r="F30" s="195" t="s">
         <v>377</v>
@@ -29066,7 +29074,7 @@
       <c r="B31" s="294" t="s">
         <v>406</v>
       </c>
-      <c r="C31" s="285"/>
+      <c r="C31" s="282"/>
       <c r="D31" s="280"/>
       <c r="F31" s="195" t="s">
         <v>380</v>
@@ -29095,7 +29103,7 @@
       <c r="B32" s="294" t="s">
         <v>407</v>
       </c>
-      <c r="C32" s="285"/>
+      <c r="C32" s="282"/>
       <c r="D32" s="280"/>
       <c r="F32" s="195" t="s">
         <v>383</v>
@@ -29116,11 +29124,11 @@
       <c r="A33" s="194" t="s">
         <v>384</v>
       </c>
-      <c r="B33" s="296" t="str">
+      <c r="B33" s="301" t="str">
         <f ca="1">IF(Scorecard!D6="","not in Events list",TEXT(Scorecard!D6,"ddd d mmm yyyy")&amp;"  —  in "&amp;(Scorecard!D6-TODAY())&amp;" days")</f>
         <v>Thu 29 Oct 2026  —  in 14 days</v>
       </c>
-      <c r="C33" s="285"/>
+      <c r="C33" s="282"/>
       <c r="D33" s="280"/>
       <c r="F33" s="195" t="s">
         <v>385</v>
@@ -29149,7 +29157,7 @@
       <c r="B34" s="294" t="s">
         <v>408</v>
       </c>
-      <c r="C34" s="285"/>
+      <c r="C34" s="282"/>
       <c r="D34" s="280"/>
       <c r="F34" s="195" t="s">
         <v>388</v>
@@ -29171,7 +29179,7 @@
       <c r="B35" s="294" t="s">
         <v>409</v>
       </c>
-      <c r="C35" s="285"/>
+      <c r="C35" s="282"/>
       <c r="D35" s="280"/>
       <c r="F35" s="195" t="s">
         <v>391</v>
@@ -29195,7 +29203,7 @@
       <c r="B36" s="294" t="s">
         <v>410</v>
       </c>
-      <c r="C36" s="285"/>
+      <c r="C36" s="282"/>
       <c r="D36" s="280"/>
       <c r="F36" s="195" t="s">
         <v>394</v>
@@ -29218,7 +29226,7 @@
       <c r="B37" s="294" t="s">
         <v>411</v>
       </c>
-      <c r="C37" s="285"/>
+      <c r="C37" s="282"/>
       <c r="D37" s="280"/>
       <c r="F37" s="195" t="s">
         <v>397</v>
@@ -29306,7 +29314,7 @@
       <c r="J42" s="208"/>
     </row>
     <row r="43" spans="1:10" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A43" s="300" t="s">
+      <c r="A43" s="299" t="s">
         <v>370</v>
       </c>
       <c r="B43" s="273"/>
@@ -29335,7 +29343,7 @@
       <c r="B44" s="294" t="s">
         <v>415</v>
       </c>
-      <c r="C44" s="285"/>
+      <c r="C44" s="282"/>
       <c r="D44" s="280"/>
       <c r="F44" s="195" t="s">
         <v>377</v>
@@ -29360,7 +29368,7 @@
       <c r="B45" s="294" t="s">
         <v>416</v>
       </c>
-      <c r="C45" s="285"/>
+      <c r="C45" s="282"/>
       <c r="D45" s="280"/>
       <c r="F45" s="195" t="s">
         <v>380</v>
@@ -29389,7 +29397,7 @@
       <c r="B46" s="294" t="s">
         <v>417</v>
       </c>
-      <c r="C46" s="285"/>
+      <c r="C46" s="282"/>
       <c r="D46" s="280"/>
       <c r="F46" s="195" t="s">
         <v>383</v>
@@ -29410,11 +29418,11 @@
       <c r="A47" s="194" t="s">
         <v>384</v>
       </c>
-      <c r="B47" s="296" t="str">
+      <c r="B47" s="301" t="str">
         <f ca="1">IF(Scorecard!D7="","not in Events list",TEXT(Scorecard!D7,"ddd d mmm yyyy")&amp;"  —  in "&amp;(Scorecard!D7-TODAY())&amp;" days")</f>
         <v>Thu 5 Nov 2026  —  in 21 days</v>
       </c>
-      <c r="C47" s="285"/>
+      <c r="C47" s="282"/>
       <c r="D47" s="280"/>
       <c r="F47" s="195" t="s">
         <v>385</v>
@@ -29443,7 +29451,7 @@
       <c r="B48" s="294" t="s">
         <v>418</v>
       </c>
-      <c r="C48" s="285"/>
+      <c r="C48" s="282"/>
       <c r="D48" s="280"/>
       <c r="F48" s="195" t="s">
         <v>388</v>
@@ -29467,7 +29475,7 @@
       <c r="B49" s="294" t="s">
         <v>419</v>
       </c>
-      <c r="C49" s="285"/>
+      <c r="C49" s="282"/>
       <c r="D49" s="280"/>
       <c r="F49" s="195" t="s">
         <v>391</v>
@@ -29491,7 +29499,7 @@
       <c r="B50" s="294" t="s">
         <v>420</v>
       </c>
-      <c r="C50" s="285"/>
+      <c r="C50" s="282"/>
       <c r="D50" s="280"/>
       <c r="F50" s="195" t="s">
         <v>394</v>
@@ -29514,7 +29522,7 @@
       <c r="B51" s="294" t="s">
         <v>421</v>
       </c>
-      <c r="C51" s="285"/>
+      <c r="C51" s="282"/>
       <c r="D51" s="280"/>
       <c r="F51" s="195" t="s">
         <v>397</v>
@@ -29602,7 +29610,7 @@
       <c r="J56" s="210"/>
     </row>
     <row r="57" spans="1:10" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A57" s="300" t="s">
+      <c r="A57" s="299" t="s">
         <v>370</v>
       </c>
       <c r="B57" s="273"/>
@@ -29631,7 +29639,7 @@
       <c r="B58" s="294" t="s">
         <v>424</v>
       </c>
-      <c r="C58" s="285"/>
+      <c r="C58" s="282"/>
       <c r="D58" s="280"/>
       <c r="F58" s="195" t="s">
         <v>377</v>
@@ -29656,7 +29664,7 @@
       <c r="B59" s="294" t="s">
         <v>425</v>
       </c>
-      <c r="C59" s="285"/>
+      <c r="C59" s="282"/>
       <c r="D59" s="280"/>
       <c r="F59" s="195" t="s">
         <v>380</v>
@@ -29685,7 +29693,7 @@
       <c r="B60" s="294" t="s">
         <v>426</v>
       </c>
-      <c r="C60" s="285"/>
+      <c r="C60" s="282"/>
       <c r="D60" s="280"/>
       <c r="F60" s="195" t="s">
         <v>383</v>
@@ -29704,11 +29712,11 @@
       <c r="A61" s="194" t="s">
         <v>384</v>
       </c>
-      <c r="B61" s="296" t="str">
+      <c r="B61" s="301" t="str">
         <f ca="1">IF(Scorecard!D8="","not in Events list",TEXT(Scorecard!D8,"ddd d mmm yyyy")&amp;"  —  in "&amp;(Scorecard!D8-TODAY())&amp;" days")</f>
         <v>Fri 30 Oct 2026  —  in 15 days</v>
       </c>
-      <c r="C61" s="285"/>
+      <c r="C61" s="282"/>
       <c r="D61" s="280"/>
       <c r="F61" s="195" t="s">
         <v>385</v>
@@ -29737,7 +29745,7 @@
       <c r="B62" s="294" t="s">
         <v>427</v>
       </c>
-      <c r="C62" s="285"/>
+      <c r="C62" s="282"/>
       <c r="D62" s="280"/>
       <c r="F62" s="195" t="s">
         <v>388</v>
@@ -29759,7 +29767,7 @@
       <c r="B63" s="294" t="s">
         <v>428</v>
       </c>
-      <c r="C63" s="285"/>
+      <c r="C63" s="282"/>
       <c r="D63" s="280"/>
       <c r="F63" s="195" t="s">
         <v>391</v>
@@ -29783,7 +29791,7 @@
       <c r="B64" s="294" t="s">
         <v>429</v>
       </c>
-      <c r="C64" s="285"/>
+      <c r="C64" s="282"/>
       <c r="D64" s="280"/>
       <c r="F64" s="195" t="s">
         <v>394</v>
@@ -29806,7 +29814,7 @@
       <c r="B65" s="294" t="s">
         <v>430</v>
       </c>
-      <c r="C65" s="285"/>
+      <c r="C65" s="282"/>
       <c r="D65" s="280"/>
       <c r="F65" s="195" t="s">
         <v>397</v>
@@ -29894,7 +29902,7 @@
       <c r="J70" s="212"/>
     </row>
     <row r="71" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A71" s="300" t="s">
+      <c r="A71" s="299" t="s">
         <v>433</v>
       </c>
       <c r="B71" s="273"/>
@@ -29953,7 +29961,7 @@
       <c r="A73" s="215"/>
       <c r="B73" s="215"/>
       <c r="C73" s="215"/>
-      <c r="D73" s="297"/>
+      <c r="D73" s="306"/>
       <c r="F73" s="213" t="s">
         <v>439</v>
       </c>
@@ -29978,7 +29986,7 @@
       <c r="A74" s="215"/>
       <c r="B74" s="215"/>
       <c r="C74" s="215"/>
-      <c r="D74" s="298"/>
+      <c r="D74" s="307"/>
       <c r="F74" s="213" t="s">
         <v>18</v>
       </c>
@@ -29999,7 +30007,7 @@
       </c>
       <c r="B75" s="188"/>
       <c r="C75" s="294"/>
-      <c r="D75" s="304"/>
+      <c r="D75" s="295"/>
       <c r="F75" s="213" t="s">
         <v>440</v>
       </c>
@@ -30017,8 +30025,8 @@
     <row r="76" spans="1:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A76" s="215"/>
       <c r="B76" s="215"/>
-      <c r="C76" s="305"/>
-      <c r="D76" s="306"/>
+      <c r="C76" s="296"/>
+      <c r="D76" s="297"/>
       <c r="F76" s="219" t="s">
         <v>441</v>
       </c>
@@ -30034,7 +30042,7 @@
       </c>
     </row>
     <row r="78" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A78" s="299" t="s">
+      <c r="A78" s="304" t="s">
         <v>442</v>
       </c>
       <c r="B78" s="273"/>
@@ -30061,6 +30069,48 @@
     </row>
   </sheetData>
   <mergeCells count="58">
+    <mergeCell ref="I6:J6"/>
+    <mergeCell ref="B23:D23"/>
+    <mergeCell ref="B61:D61"/>
+    <mergeCell ref="D72:D74"/>
+    <mergeCell ref="B17:D17"/>
+    <mergeCell ref="B51:D51"/>
+    <mergeCell ref="B64:D64"/>
+    <mergeCell ref="B20:D20"/>
+    <mergeCell ref="B33:D33"/>
+    <mergeCell ref="B36:D36"/>
+    <mergeCell ref="C67:D67"/>
+    <mergeCell ref="A78:J79"/>
+    <mergeCell ref="A29:D29"/>
+    <mergeCell ref="A4:J4"/>
+    <mergeCell ref="A43:D43"/>
+    <mergeCell ref="B44:D44"/>
+    <mergeCell ref="A10:J10"/>
+    <mergeCell ref="B34:D34"/>
+    <mergeCell ref="D6:E6"/>
+    <mergeCell ref="B19:D19"/>
+    <mergeCell ref="B37:D37"/>
+    <mergeCell ref="I7:J7"/>
+    <mergeCell ref="C25:D25"/>
+    <mergeCell ref="B49:D49"/>
+    <mergeCell ref="A15:D15"/>
+    <mergeCell ref="B30:D30"/>
+    <mergeCell ref="B65:D65"/>
+    <mergeCell ref="A1:G1"/>
+    <mergeCell ref="D7:E7"/>
+    <mergeCell ref="B45:D45"/>
+    <mergeCell ref="B63:D63"/>
+    <mergeCell ref="B32:D32"/>
+    <mergeCell ref="B50:D50"/>
+    <mergeCell ref="B35:D35"/>
+    <mergeCell ref="B21:D21"/>
+    <mergeCell ref="B60:D60"/>
+    <mergeCell ref="B46:D46"/>
+    <mergeCell ref="B22:D22"/>
+    <mergeCell ref="B18:D18"/>
+    <mergeCell ref="A12:J12"/>
+    <mergeCell ref="B58:D58"/>
+    <mergeCell ref="A57:D57"/>
     <mergeCell ref="C75:D76"/>
     <mergeCell ref="A2:J2"/>
     <mergeCell ref="C53:D53"/>
@@ -30077,48 +30127,6 @@
     <mergeCell ref="D8:E8"/>
     <mergeCell ref="B59:D59"/>
     <mergeCell ref="B31:D31"/>
-    <mergeCell ref="B46:D46"/>
-    <mergeCell ref="B22:D22"/>
-    <mergeCell ref="B18:D18"/>
-    <mergeCell ref="A12:J12"/>
-    <mergeCell ref="B58:D58"/>
-    <mergeCell ref="A57:D57"/>
-    <mergeCell ref="A1:G1"/>
-    <mergeCell ref="D7:E7"/>
-    <mergeCell ref="B45:D45"/>
-    <mergeCell ref="B63:D63"/>
-    <mergeCell ref="B32:D32"/>
-    <mergeCell ref="B50:D50"/>
-    <mergeCell ref="B35:D35"/>
-    <mergeCell ref="B21:D21"/>
-    <mergeCell ref="A78:J79"/>
-    <mergeCell ref="A29:D29"/>
-    <mergeCell ref="A4:J4"/>
-    <mergeCell ref="A43:D43"/>
-    <mergeCell ref="B44:D44"/>
-    <mergeCell ref="A10:J10"/>
-    <mergeCell ref="B34:D34"/>
-    <mergeCell ref="D6:E6"/>
-    <mergeCell ref="B19:D19"/>
-    <mergeCell ref="B37:D37"/>
-    <mergeCell ref="I7:J7"/>
-    <mergeCell ref="C25:D25"/>
-    <mergeCell ref="B49:D49"/>
-    <mergeCell ref="A15:D15"/>
-    <mergeCell ref="B30:D30"/>
-    <mergeCell ref="B65:D65"/>
-    <mergeCell ref="B60:D60"/>
-    <mergeCell ref="I6:J6"/>
-    <mergeCell ref="B23:D23"/>
-    <mergeCell ref="B61:D61"/>
-    <mergeCell ref="D72:D74"/>
-    <mergeCell ref="B17:D17"/>
-    <mergeCell ref="B51:D51"/>
-    <mergeCell ref="B64:D64"/>
-    <mergeCell ref="B20:D20"/>
-    <mergeCell ref="B33:D33"/>
-    <mergeCell ref="B36:D36"/>
-    <mergeCell ref="C67:D67"/>
   </mergeCells>
   <conditionalFormatting sqref="B24:B25">
     <cfRule type="expression" dxfId="171" priority="13" stopIfTrue="1">
@@ -30823,12 +30831,12 @@
         <f>L4&amp;" wins "&amp;COUNTIF(G5:G11,L4)&amp;" of 7, "&amp;L5&amp;" wins "&amp;COUNTIF(G5:G11,L5)&amp;", level on "&amp;COUNTIF(G5:G11,"LEVEL")</f>
         <v>USD wins 1 of 7, GBP wins 0, level on 6</v>
       </c>
-      <c r="C16" s="285"/>
-      <c r="D16" s="285"/>
-      <c r="E16" s="285"/>
-      <c r="F16" s="285"/>
-      <c r="G16" s="285"/>
-      <c r="H16" s="285"/>
+      <c r="C16" s="282"/>
+      <c r="D16" s="282"/>
+      <c r="E16" s="282"/>
+      <c r="F16" s="282"/>
+      <c r="G16" s="282"/>
+      <c r="H16" s="282"/>
       <c r="I16" s="280"/>
       <c r="J16" s="7"/>
       <c r="K16" s="7"/>
@@ -30842,12 +30850,12 @@
         <f>IF(L9="","No directional call — use as comparison only",IF(COUNTIF(H5:H11,"BACKS THE CALL")&gt;=5,"STRONG — evidence backs the call",IF(COUNTIF(H5:H11,"BACKS THE CALL")&gt;COUNTIF(H5:H11,"AGAINST"),"MODERATE — more for than against","WEAK — evidence does not back the call")))</f>
         <v>No directional call — use as comparison only</v>
       </c>
-      <c r="C17" s="285"/>
-      <c r="D17" s="285"/>
-      <c r="E17" s="285"/>
-      <c r="F17" s="285"/>
-      <c r="G17" s="285"/>
-      <c r="H17" s="285"/>
+      <c r="C17" s="282"/>
+      <c r="D17" s="282"/>
+      <c r="E17" s="282"/>
+      <c r="F17" s="282"/>
+      <c r="G17" s="282"/>
+      <c r="H17" s="282"/>
       <c r="I17" s="280"/>
       <c r="J17" s="7"/>
       <c r="K17" s="7"/>
@@ -30861,12 +30869,12 @@
         <f>IF(MAX(F5:F8)&gt;0,INDEX(A5:A8,MATCH(MAX(F5:F8),F5:F8,0))&amp;"  (gap +"&amp;MAX(F5:F8)&amp;")","None in the four scores")</f>
         <v>None in the four scores</v>
       </c>
-      <c r="C18" s="285"/>
-      <c r="D18" s="285"/>
-      <c r="E18" s="285"/>
-      <c r="F18" s="285"/>
-      <c r="G18" s="285"/>
-      <c r="H18" s="285"/>
+      <c r="C18" s="282"/>
+      <c r="D18" s="282"/>
+      <c r="E18" s="282"/>
+      <c r="F18" s="282"/>
+      <c r="G18" s="282"/>
+      <c r="H18" s="282"/>
       <c r="I18" s="280"/>
       <c r="J18" s="7"/>
       <c r="K18" s="7"/>
@@ -30880,12 +30888,12 @@
         <f>IF(MIN(F5:F8)&lt;0,INDEX(A5:A8,MATCH(MIN(F5:F8),F5:F8,0))&amp;"  (gap "&amp;MIN(F5:F8)&amp;")","None in the four scores")</f>
         <v>None in the four scores</v>
       </c>
-      <c r="C19" s="285"/>
-      <c r="D19" s="285"/>
-      <c r="E19" s="285"/>
-      <c r="F19" s="285"/>
-      <c r="G19" s="285"/>
-      <c r="H19" s="285"/>
+      <c r="C19" s="282"/>
+      <c r="D19" s="282"/>
+      <c r="E19" s="282"/>
+      <c r="F19" s="282"/>
+      <c r="G19" s="282"/>
+      <c r="H19" s="282"/>
       <c r="I19" s="280"/>
       <c r="J19" s="7"/>
       <c r="K19" s="7"/>
@@ -30898,12 +30906,12 @@
       <c r="B20" s="310" t="s">
         <v>477</v>
       </c>
-      <c r="C20" s="285"/>
-      <c r="D20" s="285"/>
-      <c r="E20" s="285"/>
-      <c r="F20" s="285"/>
-      <c r="G20" s="285"/>
-      <c r="H20" s="285"/>
+      <c r="C20" s="282"/>
+      <c r="D20" s="282"/>
+      <c r="E20" s="282"/>
+      <c r="F20" s="282"/>
+      <c r="G20" s="282"/>
+      <c r="H20" s="282"/>
       <c r="I20" s="280"/>
       <c r="J20" s="7"/>
       <c r="K20" s="7"/>
@@ -30916,12 +30924,12 @@
       <c r="B21" s="310" t="s">
         <v>479</v>
       </c>
-      <c r="C21" s="285"/>
-      <c r="D21" s="285"/>
-      <c r="E21" s="285"/>
-      <c r="F21" s="285"/>
-      <c r="G21" s="285"/>
-      <c r="H21" s="285"/>
+      <c r="C21" s="282"/>
+      <c r="D21" s="282"/>
+      <c r="E21" s="282"/>
+      <c r="F21" s="282"/>
+      <c r="G21" s="282"/>
+      <c r="H21" s="282"/>
       <c r="I21" s="280"/>
       <c r="J21" s="7"/>
       <c r="K21" s="7"/>
@@ -40064,7 +40072,7 @@
         <v>620</v>
       </c>
     </row>
-    <row r="13" spans="1:6" ht="33.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:6" ht="36.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="82" t="s">
         <v>621</v>
       </c>
@@ -40126,7 +40134,7 @@
         <v>625</v>
       </c>
     </row>
-    <row r="16" spans="1:6" ht="37.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:6" ht="51.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="82" t="s">
         <v>626</v>
       </c>
@@ -40244,8 +40252,8 @@
     <col min="8" max="8" width="14.7109375" customWidth="1"/>
     <col min="9" max="9" width="13" customWidth="1"/>
     <col min="10" max="10" width="26" customWidth="1"/>
-    <col min="11" max="11" width="12" customWidth="1"/>
-    <col min="12" max="12" width="16" customWidth="1"/>
+    <col min="11" max="11" width="16" customWidth="1"/>
+    <col min="12" max="12" width="18.140625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:12" ht="33.950000000000003" customHeight="1" x14ac:dyDescent="0.25">

</xml_diff>